<commit_message>
Complete three-entity exam center for defense
</commit_message>
<xml_diff>
--- a/outputs/exam-center/from_database.xlsx
+++ b/outputs/exam-center/from_database.xlsx
@@ -8,16 +8,18 @@
   <sheets>
     <sheet name="Кандидаты" r:id="rId3" sheetId="1"/>
     <sheet name="Заявки" r:id="rId4" sheetId="2"/>
+    <sheet name="Экзаменаторы" r:id="rId5" sheetId="3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Кандидаты!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Кандидаты!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Заявки!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="true">Экзаменаторы!$A$1:$E$1</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="53">
   <si>
     <t>ID</t>
   </si>
@@ -31,6 +33,9 @@
     <t>Телефон</t>
   </si>
   <si>
+    <t>Статус</t>
+  </si>
+  <si>
     <t>Анна Смирнова</t>
   </si>
   <si>
@@ -40,6 +45,9 @@
     <t>+7 900 111-11-11</t>
   </si>
   <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
     <t>Борис Иванов</t>
   </si>
   <si>
@@ -88,9 +96,6 @@
     <t>Дата экзамена</t>
   </si>
   <si>
-    <t>Статус</t>
-  </si>
-  <si>
     <t>Балл</t>
   </si>
   <si>
@@ -137,6 +142,42 @@
   </si>
   <si>
     <t>Математика</t>
+  </si>
+  <si>
+    <t>Предмет</t>
+  </si>
+  <si>
+    <t>Мария Петрова</t>
+  </si>
+  <si>
+    <t>maria.petrova@exam.org</t>
+  </si>
+  <si>
+    <t>Игорь Волков</t>
+  </si>
+  <si>
+    <t>igor.volkov@exam.org</t>
+  </si>
+  <si>
+    <t>Елена Морозова</t>
+  </si>
+  <si>
+    <t>elena.morozova@exam.org</t>
+  </si>
+  <si>
+    <t>Ольга Белова</t>
+  </si>
+  <si>
+    <t>olga.belova@exam.org</t>
+  </si>
+  <si>
+    <t>INACTIVE</t>
+  </si>
+  <si>
+    <t>Павел Романов</t>
+  </si>
+  <si>
+    <t>pavel.romanov@exam.org</t>
   </si>
 </sst>
 </file>
@@ -201,13 +242,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.0" customWidth="true"/>
     <col min="2" max="2" width="30.0" customWidth="true"/>
     <col min="3" max="3" width="34.0" customWidth="true"/>
     <col min="4" max="4" width="22.0" customWidth="true"/>
+    <col min="5" max="5" width="16.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -223,19 +265,25 @@
       <c r="D1" t="s" s="1">
         <v>3</v>
       </c>
+      <c r="E1" t="s" s="1">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -243,13 +291,16 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -257,13 +308,16 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -271,13 +325,16 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -285,17 +342,20 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:E1"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
@@ -321,28 +381,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="1">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s" s="1">
         <v>2</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F1" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G1" t="s" s="1">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -353,19 +413,19 @@
         <v>2.0</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F2" t="n" s="2">
         <v>46284.833333333336</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H2" t="n" s="0">
         <v>87.0</v>
@@ -382,19 +442,19 @@
         <v>1.0</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" t="n" s="2">
         <v>46301.833333333336</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I3" t="n" s="2">
         <v>46289.84424818287</v>
@@ -408,19 +468,19 @@
         <v>2.0</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F4" t="n" s="2">
         <v>46293.833333333336</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I4" t="n" s="2">
         <v>46289.84424818287</v>
@@ -434,19 +494,19 @@
         <v>3.0</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F5" t="n" s="2">
         <v>46298.833333333336</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I5" t="n" s="2">
         <v>46289.84424818287</v>
@@ -460,19 +520,19 @@
         <v>4.0</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F6" t="n" s="2">
         <v>46304.833333333336</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" t="n" s="2">
         <v>46289.84424818287</v>
@@ -486,19 +546,19 @@
         <v>4.0</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F7" t="n" s="2">
         <v>46305.833333333336</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I7" t="n" s="2">
         <v>46289.84424818287</v>
@@ -512,19 +572,19 @@
         <v>5.0</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F8" t="n" s="2">
         <v>46287.833333333336</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I8" t="n" s="2">
         <v>46289.84424818287</v>
@@ -538,19 +598,19 @@
         <v>5.0</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F9" t="n" s="2">
         <v>46309.833333333336</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I9" t="n" s="2">
         <v>46289.84424818287</v>
@@ -564,19 +624,19 @@
         <v>3.0</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F10" t="n" s="2">
         <v>46281.833333333336</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H10" t="n" s="0">
         <v>74.0</v>
@@ -593,19 +653,19 @@
         <v>1.0</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F11" t="n" s="2">
         <v>46296.833333333336</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I11" t="n" s="2">
         <v>46289.84424818287</v>
@@ -615,4 +675,124 @@
   <autoFilter ref="A1:I1"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="10.0" customWidth="true"/>
+    <col min="2" max="2" width="30.0" customWidth="true"/>
+    <col min="3" max="3" width="34.0" customWidth="true"/>
+    <col min="4" max="4" width="25.0" customWidth="true"/>
+    <col min="5" max="5" width="16.0" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="1">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="1">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>